<commit_message>
Formats of the APA tables and figures, the common test, and Word (v0.10, step 3, D-082 to D-085)
A format renders the neutral description and reads its own text back; FORMATS lists them,
for the page and the command line. The common test renders every analysis and option, in
French and English, in every registered format, and finds every header, cell, title and
note in the file, and a person's edits. Word: real tables with APA rules only, numbers that
never wrap, figures as images drawn once for every format (matplotlib), checked in Word.
python-docx and matplotlib are new dependencies. python-docx brings lxml, which openpyxl
then uses: the example Excel files are regenerated, their cells unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011aKk4abgDh4Wf3T24BCG72
</commit_message>
<xml_diff>
--- a/exemples/bases-fictives/etude-sommeil.xlsx
+++ b/exemples/bases-fictives/etude-sommeil.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="donnees" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="donnees" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>